<commit_message>
Add dashboard alumni and mobile app support
</commit_message>
<xml_diff>
--- a/PRATIBHA_BULK_USERS_TEMPLATE.xlsx
+++ b/PRATIBHA_BULK_USERS_TEMPLATE.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,24 +26,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000F172A"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -60,9 +56,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,14 +422,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -551,6 +545,35 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Aman Alumni</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>amanalumni</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ChangeMe123</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>alumni</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Alumni Mentor</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>